<commit_message>
Improving readability of slides by changing font color + better coverage of descendant's role
</commit_message>
<xml_diff>
--- a/results/ate_evalue_survey.xlsx
+++ b/results/ate_evalue_survey.xlsx
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4385066466877225</v>
+        <v>0.4385066466877226</v>
       </c>
       <c r="D2" t="n">
         <v>1.490394795801431</v>
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.0003080184020601404</v>
+        <v>-0.0003080184020606004</v>
       </c>
       <c r="D3" t="n">
-        <v>1.000280336032678</v>
+        <v>1.000280336032679</v>
       </c>
       <c r="E3" t="n">
-        <v>1.017025921151431</v>
+        <v>1.017025921151445</v>
       </c>
       <c r="F3" t="n">
         <v>1.433204662544642</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.9472230553604767</v>
+        <v>0.9472230553604785</v>
       </c>
       <c r="J3" t="b">
         <v>0</v>
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1560165140786423</v>
+        <v>0.1560165140786419</v>
       </c>
       <c r="D4" t="n">
-        <v>1.152547866535128</v>
+        <v>1.152547866535127</v>
       </c>
       <c r="E4" t="n">
-        <v>1.571855293275398</v>
+        <v>1.571855293275396</v>
       </c>
       <c r="F4" t="n">
         <v>1.381038924028185</v>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>7.251803917655306e-05</v>
+        <v>7.251803917655267e-05</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Rerunning diagram generation + manual update
</commit_message>
<xml_diff>
--- a/results/ate_evalue_survey.xlsx
+++ b/results/ate_evalue_survey.xlsx
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>4.491231826565502e-25</v>
+        <v>4.491231826565693e-25</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.00538806080623125</v>
+        <v>-0.005388060806230331</v>
       </c>
       <c r="D3" t="n">
-        <v>1.004915175371656</v>
+        <v>1.004915175371655</v>
       </c>
       <c r="E3" t="n">
-        <v>1.075195573211952</v>
+        <v>1.075195573211946</v>
       </c>
       <c r="F3" t="n">
         <v>1.432806872361067</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.8572422817678189</v>
+        <v>0.8572422817678169</v>
       </c>
       <c r="J3" t="b">
         <v>0</v>
@@ -572,13 +572,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.163544348696728</v>
+        <v>0.163544348696727</v>
       </c>
       <c r="D4" t="n">
-        <v>1.160470303859981</v>
+        <v>1.16047030385998</v>
       </c>
       <c r="E4" t="n">
-        <v>1.592003642410892</v>
+        <v>1.592003642410889</v>
       </c>
       <c r="F4" t="n">
         <v>1.383351419900095</v>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>0.0001393008282982229</v>
+        <v>0.0001393008282982222</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Clarify IPTW framing: not formally doubly robust
</commit_message>
<xml_diff>
--- a/results/ate_evalue_survey.xlsx
+++ b/results/ate_evalue_survey.xlsx
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.4731872093428421</v>
+        <v>0.4731872093428426</v>
       </c>
       <c r="D2" t="n">
-        <v>1.538180709341215</v>
+        <v>1.538180709341216</v>
       </c>
       <c r="E2" t="n">
-        <v>2.448026402438802</v>
+        <v>2.448026402438805</v>
       </c>
       <c r="F2" t="n">
         <v>2.182214874657829</v>
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>4.491231826565693e-25</v>
+        <v>4.491231826565276e-25</v>
       </c>
       <c r="J2" t="b">
         <v>1</v>
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.00538806080623125</v>
+        <v>-0.005388060806230791</v>
       </c>
       <c r="D3" t="n">
         <v>1.004915175371656</v>
       </c>
       <c r="E3" t="n">
-        <v>1.075195573211952</v>
+        <v>1.07519557321195</v>
       </c>
       <c r="F3" t="n">
         <v>1.432806872361067</v>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.8572422817678174</v>
+        <v>0.8572422817678194</v>
       </c>
       <c r="J3" t="b">
         <v>0</v>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>0.0001393008282982222</v>
+        <v>0.0001393008282982229</v>
       </c>
       <c r="J4" t="b">
         <v>1</v>

</xml_diff>